<commit_message>
fix(lease-comps): Round 76gn.n — drop Subject Excel table (Excel rejects writeBuffer output)
</commit_message>
<xml_diff>
--- a/assets/cm-templates/dialysis-lease-comps-template.xlsx
+++ b/assets/cm-templates/dialysis-lease-comps-template.xlsx
@@ -338,38 +338,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Subject" displayName="Subject" ref="B3:W4" headerRowCount="1">
-  <autoFilter ref="B3:W4"/>
-  <tableColumns count="22">
-    <tableColumn id="2" name="TENANT"/>
-    <tableColumn id="3" name="OPERATOR"/>
-    <tableColumn id="4" name="ADDRESS"/>
-    <tableColumn id="5" name="CITY"/>
-    <tableColumn id="6" name="STATE"/>
-    <tableColumn id="7" name="LAND"/>
-    <tableColumn id="8" name="BUILT"/>
-    <tableColumn id="9" name="RENOVATED"/>
-    <tableColumn id="10" name="RBA"/>
-    <tableColumn id="11" name="SF LEASED"/>
-    <tableColumn id="12" name="OCCUPANCY"/>
-    <tableColumn id="13" name="RENT/SF"/>
-    <tableColumn id="14" name="CURRENT RENT"/>
-    <tableColumn id="15" name="COMMENCE"/>
-    <tableColumn id="16" name="EXP"/>
-    <tableColumn id="17" name="INITIAL TERM"/>
-    <tableColumn id="18" name="TERM REM"/>
-    <tableColumn id="19" name="EXPENSES"/>
-    <tableColumn id="20" name="BUMPS"/>
-    <tableColumn id="21" name="USER/OWNER"/>
-    <tableColumn id="22" name="DISTANCE TO SUBJECT"/>
-    <tableColumn id="23" name="PATIENTS"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Comps" displayName="Comps" ref="B7:W60" headerRowCount="1" totalsRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Comps" displayName="Comps" ref="B7:W60" headerRowCount="1" totalsRowCount="1">
   <autoFilter ref="B7:W60"/>
   <tableColumns count="22">
     <tableColumn id="2" name="TENANT"/>
@@ -2060,9 +2029,8 @@
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <tableParts count="2">
+  <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
regen lease-comps template binary (Round 76gn.q — ST/RENO/COMM headers)
</commit_message>
<xml_diff>
--- a/assets/cm-templates/dialysis-lease-comps-template.xlsx
+++ b/assets/cm-templates/dialysis-lease-comps-template.xlsx
@@ -345,16 +345,16 @@
     <tableColumn id="3" name="OPERATOR"/>
     <tableColumn id="4" name="ADDRESS"/>
     <tableColumn id="5" name="CITY"/>
-    <tableColumn id="6" name="STATE"/>
+    <tableColumn id="6" name="ST"/>
     <tableColumn id="7" name="LAND"/>
     <tableColumn id="8" name="BUILT"/>
-    <tableColumn id="9" name="RENOVATED"/>
+    <tableColumn id="9" name="RENO"/>
     <tableColumn id="10" name="RBA"/>
     <tableColumn id="11" name="SF LEASED"/>
     <tableColumn id="12" name="OCCUPANCY"/>
     <tableColumn id="13" name="RENT/SF"/>
     <tableColumn id="14" name="CURRENT RENT"/>
-    <tableColumn id="15" name="COMMENCE"/>
+    <tableColumn id="15" name="COMM"/>
     <tableColumn id="16" name="EXP"/>
     <tableColumn id="17" name="INITIAL TERM"/>
     <tableColumn id="18" name="TERM REM"/>
@@ -770,7 +770,7 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>STATE</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>RENOVATED</t>
+          <t>RENO</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="O3" s="6" t="inlineStr">
         <is>
-          <t>COMMENCE</t>
+          <t>COMM</t>
         </is>
       </c>
       <c r="P3" s="6" t="inlineStr">
@@ -943,7 +943,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>STATE</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -958,7 +958,7 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>RENOVATED</t>
+          <t>RENO</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
-          <t>COMMENCE</t>
+          <t>COMM</t>
         </is>
       </c>
       <c r="P7" s="6" t="inlineStr">
@@ -1974,7 +1974,7 @@
         <v/>
       </c>
       <c r="I60" s="35">
-        <f>IFERROR(SUBTOTAL(101,Comps[RENOVATED]),"")</f>
+        <f>IFERROR(SUBTOTAL(101,Comps[RENO]),"")</f>
         <v/>
       </c>
       <c r="J60" s="36">

</xml_diff>